<commit_message>
add vendas_sac field, 3 sales charts per category, zero-fill missing days
Agent-Logs-Url: https://github.com/ecommerce-b2pro/dashboardB2/sessions/88e49475-0c72-4638-8dba-086160593708

Co-authored-by: ecommerce-b2pro <271341905+ecommerce-b2pro@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/exemplo_importacao.xlsx
+++ b/exemplo_importacao.xlsx
@@ -397,12 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:F11"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -413,10 +415,16 @@
         <v>ecommerce</v>
       </c>
       <c r="C1" t="str">
-        <v>quantidade</v>
+        <v>vendas_ecommerce</v>
       </c>
       <c r="D1" t="str">
-        <v>receita</v>
+        <v>receita_ecommerce</v>
+      </c>
+      <c r="E1" t="str">
+        <v>vendas_sac</v>
+      </c>
+      <c r="F1" t="str">
+        <v>receita_sac</v>
       </c>
     </row>
     <row r="2">
@@ -432,6 +440,12 @@
       <c r="D2">
         <v>1200</v>
       </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2">
+        <v>120</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -446,6 +460,12 @@
       <c r="D3">
         <v>800</v>
       </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>80</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -460,6 +480,12 @@
       <c r="D4">
         <v>1440</v>
       </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <v>144</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -474,6 +500,12 @@
       <c r="D5">
         <v>600</v>
       </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>60</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -488,6 +520,12 @@
       <c r="D6">
         <v>1500</v>
       </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>150</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -502,6 +540,12 @@
       <c r="D7">
         <v>2160</v>
       </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7">
+        <v>216</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -516,6 +560,12 @@
       <c r="D8">
         <v>900</v>
       </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>90</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -530,6 +580,12 @@
       <c r="D9">
         <v>1100</v>
       </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>110</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -544,6 +600,12 @@
       <c r="D10">
         <v>1680</v>
       </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>168</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -558,10 +620,16 @@
       <c r="D11">
         <v>700</v>
       </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>70</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>